<commit_message>
regenerate outputs with corrected sheet and CO2 partitioning
Full pipeline run against the metadata sheet as edited on 2026-10-27:
fluxes for the re-timed windows, Dark condition label, room-air flag,
and the new CO2_partitioning table and figures.
</commit_message>
<xml_diff>
--- a/output/tables/chamber_window_temperature.xlsx
+++ b/output/tables/chamber_window_temperature.xlsx
@@ -469,7 +469,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-04-01 12:35:30</t>
+          <t>2026-04-01 12:45:30</t>
         </is>
       </c>
       <c r="G37">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2569,7 +2569,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3409,7 +3409,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3493,7 +3493,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3745,7 +3745,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3829,7 +3829,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3997,7 +3997,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4165,7 +4165,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4417,7 +4417,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4501,7 +4501,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4585,7 +4585,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4753,7 +4753,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4837,7 +4837,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -4921,7 +4921,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5005,7 +5005,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5089,7 +5089,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5173,7 +5173,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5220,16 +5220,16 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2026-04-12 13:36:50</t>
+          <t>2026-04-12 13:46:50</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>2026-04-12 13:46:50</t>
+          <t>2026-04-12 13:56:50</t>
         </is>
       </c>
       <c r="G116">
-        <v>26.65405</v>
+        <v>26.654</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
@@ -5237,10 +5237,10 @@
         </is>
       </c>
       <c r="I116">
-        <v>24.99954</v>
+        <v>23.44369</v>
       </c>
       <c r="J116">
-        <v>26.67949</v>
+        <v>26.67647</v>
       </c>
     </row>
     <row r="117">
@@ -5257,21 +5257,21 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>2026-04-12 13:48:00</t>
+          <t>2026-04-12 13:58:00</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-04-12 13:58:00</t>
+          <t>2026-04-12 14:08:00</t>
         </is>
       </c>
       <c r="G117">
-        <v>26.654</v>
+        <v>26.66025</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
@@ -5279,10 +5279,10 @@
         </is>
       </c>
       <c r="I117">
-        <v>23.44369</v>
+        <v>25.49772</v>
       </c>
       <c r="J117">
-        <v>26.67647</v>
+        <v>26.68175</v>
       </c>
     </row>
     <row r="118">
@@ -5341,7 +5341,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5425,7 +5425,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5593,7 +5593,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -5761,7 +5761,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5845,7 +5845,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -5929,7 +5929,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -6013,7 +6013,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -6097,7 +6097,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -6181,7 +6181,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -6265,7 +6265,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -6349,7 +6349,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -6517,7 +6517,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -6601,7 +6601,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -6685,7 +6685,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -6769,7 +6769,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -6937,7 +6937,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -7105,7 +7105,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -7189,7 +7189,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -7273,7 +7273,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -7357,7 +7357,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -7441,7 +7441,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -7525,7 +7525,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -7609,7 +7609,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
@@ -7693,7 +7693,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -7777,7 +7777,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -7861,7 +7861,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
@@ -7945,7 +7945,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -8029,7 +8029,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -8113,7 +8113,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
@@ -8197,7 +8197,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -8281,7 +8281,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
@@ -8365,7 +8365,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
@@ -8449,7 +8449,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
@@ -8533,7 +8533,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
@@ -8617,7 +8617,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
@@ -8701,7 +8701,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
@@ -8785,7 +8785,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -8869,7 +8869,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
@@ -9037,7 +9037,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
@@ -9121,7 +9121,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
@@ -9205,7 +9205,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
@@ -9289,7 +9289,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
@@ -9457,7 +9457,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
@@ -9541,7 +9541,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
@@ -9625,7 +9625,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
@@ -9709,7 +9709,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -9793,7 +9793,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
@@ -9877,7 +9877,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
@@ -9961,7 +9961,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
@@ -10045,7 +10045,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
@@ -10129,7 +10129,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -10213,7 +10213,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
@@ -10297,7 +10297,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
@@ -10381,7 +10381,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
@@ -10465,7 +10465,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
@@ -10549,7 +10549,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
@@ -10633,7 +10633,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
@@ -10717,7 +10717,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
@@ -10801,7 +10801,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
@@ -10885,7 +10885,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
@@ -10969,7 +10969,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -11053,7 +11053,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -11137,7 +11137,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -11221,7 +11221,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
@@ -11305,7 +11305,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
@@ -11389,7 +11389,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
@@ -11473,7 +11473,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
@@ -11557,7 +11557,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
@@ -11641,7 +11641,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
@@ -11725,7 +11725,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
@@ -11809,7 +11809,7 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
@@ -11893,7 +11893,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
@@ -11977,7 +11977,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -12061,7 +12061,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -12145,7 +12145,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -12229,7 +12229,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -12313,7 +12313,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -12397,7 +12397,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -12481,7 +12481,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -12565,7 +12565,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -12649,7 +12649,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -12733,7 +12733,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -12817,7 +12817,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -12901,7 +12901,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -12985,7 +12985,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -13069,7 +13069,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -13153,7 +13153,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -13237,7 +13237,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -13321,7 +13321,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -13405,7 +13405,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -13489,7 +13489,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -13573,7 +13573,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -13657,7 +13657,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -13741,7 +13741,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -13825,7 +13825,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -13909,7 +13909,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -13993,7 +13993,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -14077,7 +14077,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -14161,7 +14161,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -14245,7 +14245,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -14329,7 +14329,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -14413,7 +14413,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -14497,7 +14497,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -14581,7 +14581,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -14665,7 +14665,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -14749,7 +14749,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E343" t="inlineStr">
@@ -14833,7 +14833,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
@@ -14917,7 +14917,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
@@ -15001,7 +15001,7 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
@@ -15085,7 +15085,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E351" t="inlineStr">
@@ -15169,7 +15169,7 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
@@ -15337,7 +15337,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
@@ -15421,7 +15421,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -15505,7 +15505,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -15583,7 +15583,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
@@ -15655,7 +15655,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
@@ -15727,7 +15727,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
@@ -15799,7 +15799,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E369" t="inlineStr">
@@ -15871,7 +15871,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
@@ -15943,7 +15943,7 @@
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E373" t="inlineStr">
@@ -16015,7 +16015,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E375" t="inlineStr">
@@ -16056,7 +16056,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>2026-04-30 13:21:00</t>
+          <t>2026-04-30 13:12:00</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
@@ -16065,7 +16065,7 @@
         </is>
       </c>
       <c r="G376">
-        <v>26.65985230496454</v>
+        <v>26.14492173913044</v>
       </c>
       <c r="H376" t="inlineStr">
         <is>
@@ -16087,7 +16087,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E377" t="inlineStr">
@@ -16159,7 +16159,7 @@
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E379" t="inlineStr">
@@ -16231,7 +16231,7 @@
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E381" t="inlineStr">
@@ -16303,7 +16303,7 @@
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E383" t="inlineStr">
@@ -16375,7 +16375,7 @@
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E385" t="inlineStr">
@@ -16447,7 +16447,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
@@ -16519,7 +16519,7 @@
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E389" t="inlineStr">
@@ -16591,7 +16591,7 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
@@ -16663,7 +16663,7 @@
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E393" t="inlineStr">
@@ -16735,7 +16735,7 @@
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E395" t="inlineStr">
@@ -16807,7 +16807,7 @@
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E397" t="inlineStr">
@@ -16879,7 +16879,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E399" t="inlineStr">
@@ -16951,7 +16951,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E401" t="inlineStr">
@@ -16961,11 +16961,11 @@
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>2026-05-03 12:05:40</t>
+          <t>2026-05-03 13:05:40</t>
         </is>
       </c>
       <c r="G401">
-        <v>24.35780666666667</v>
+        <v>25.42964222222222</v>
       </c>
       <c r="H401" t="inlineStr">
         <is>
@@ -17023,7 +17023,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E403" t="inlineStr">
@@ -17095,7 +17095,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E405" t="inlineStr">
@@ -17167,7 +17167,7 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E407" t="inlineStr">
@@ -17239,7 +17239,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E409" t="inlineStr">
@@ -17249,11 +17249,11 @@
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>2026-05-03 10:41:05</t>
+          <t>2026-05-03 14:41:05</t>
         </is>
       </c>
       <c r="G409">
-        <v>24.45129833333333</v>
+        <v>24.80382333333333</v>
       </c>
       <c r="H409" t="inlineStr">
         <is>
@@ -17311,7 +17311,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E411" t="inlineStr">
@@ -17383,7 +17383,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E413" t="inlineStr">
@@ -17455,7 +17455,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E415" t="inlineStr">
@@ -17527,7 +17527,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E417" t="inlineStr">
@@ -17599,7 +17599,7 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E419" t="inlineStr">
@@ -17671,7 +17671,7 @@
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E421" t="inlineStr">
@@ -17743,7 +17743,7 @@
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E423" t="inlineStr">
@@ -17815,7 +17815,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E425" t="inlineStr">
@@ -17887,7 +17887,7 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E427" t="inlineStr">
@@ -17959,7 +17959,7 @@
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E429" t="inlineStr">
@@ -18031,7 +18031,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E431" t="inlineStr">
@@ -18103,7 +18103,7 @@
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E433" t="inlineStr">
@@ -18175,7 +18175,7 @@
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E435" t="inlineStr">
@@ -18247,7 +18247,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E437" t="inlineStr">
@@ -18319,7 +18319,7 @@
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E439" t="inlineStr">
@@ -18391,7 +18391,7 @@
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E441" t="inlineStr">
@@ -18463,7 +18463,7 @@
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E443" t="inlineStr">
@@ -18535,7 +18535,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E445" t="inlineStr">
@@ -18607,7 +18607,7 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E447" t="inlineStr">
@@ -18679,7 +18679,7 @@
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E449" t="inlineStr">
@@ -18751,7 +18751,7 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E451" t="inlineStr">
@@ -18823,7 +18823,7 @@
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E453" t="inlineStr">
@@ -18895,7 +18895,7 @@
       </c>
       <c r="D455" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E455" t="inlineStr">
@@ -18936,16 +18936,16 @@
       </c>
       <c r="E456" t="inlineStr">
         <is>
-          <t>2026-05-06 14:40:55</t>
+          <t>2026-05-06 15:40:55</t>
         </is>
       </c>
       <c r="F456" t="inlineStr">
         <is>
-          <t>2026-05-06 14:50:55</t>
+          <t>2026-05-06 15:50:55</t>
         </is>
       </c>
       <c r="G456">
-        <v>26.66519417989418</v>
+        <v>26.55705</v>
       </c>
       <c r="H456" t="inlineStr">
         <is>
@@ -18967,7 +18967,7 @@
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E457" t="inlineStr">
@@ -19039,7 +19039,7 @@
       </c>
       <c r="D459" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E459" t="inlineStr">
@@ -19111,7 +19111,7 @@
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E461" t="inlineStr">
@@ -19183,7 +19183,7 @@
       </c>
       <c r="D463" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E463" t="inlineStr">
@@ -19255,7 +19255,7 @@
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E465" t="inlineStr">
@@ -19327,7 +19327,7 @@
       </c>
       <c r="D467" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E467" t="inlineStr">
@@ -19399,7 +19399,7 @@
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E469" t="inlineStr">
@@ -19471,7 +19471,7 @@
       </c>
       <c r="D471" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E471" t="inlineStr">
@@ -19543,7 +19543,7 @@
       </c>
       <c r="D473" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E473" t="inlineStr">
@@ -19615,7 +19615,7 @@
       </c>
       <c r="D475" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E475" t="inlineStr">
@@ -19687,7 +19687,7 @@
       </c>
       <c r="D477" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E477" t="inlineStr">
@@ -19759,7 +19759,7 @@
       </c>
       <c r="D479" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E479" t="inlineStr">
@@ -19831,7 +19831,7 @@
       </c>
       <c r="D481" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E481" t="inlineStr">
@@ -19903,7 +19903,7 @@
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E483" t="inlineStr">
@@ -19975,7 +19975,7 @@
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E485" t="inlineStr">
@@ -20047,7 +20047,7 @@
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E487" t="inlineStr">
@@ -20119,7 +20119,7 @@
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E489" t="inlineStr">
@@ -20191,7 +20191,7 @@
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E491" t="inlineStr">
@@ -20263,7 +20263,7 @@
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E493" t="inlineStr">
@@ -20335,7 +20335,7 @@
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E495" t="inlineStr">
@@ -20407,7 +20407,7 @@
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E497" t="inlineStr">
@@ -20479,7 +20479,7 @@
       </c>
       <c r="D499" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E499" t="inlineStr">
@@ -20551,7 +20551,7 @@
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E501" t="inlineStr">
@@ -20623,7 +20623,7 @@
       </c>
       <c r="D503" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E503" t="inlineStr">
@@ -20695,7 +20695,7 @@
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E505" t="inlineStr">
@@ -20767,7 +20767,7 @@
       </c>
       <c r="D507" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E507" t="inlineStr">
@@ -20839,7 +20839,7 @@
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E509" t="inlineStr">
@@ -20911,7 +20911,7 @@
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E511" t="inlineStr">
@@ -20983,7 +20983,7 @@
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E513" t="inlineStr">
@@ -21055,7 +21055,7 @@
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E515" t="inlineStr">
@@ -21127,21 +21127,21 @@
       </c>
       <c r="D517" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E517" t="inlineStr">
         <is>
-          <t>2026-05-11 09:32:00</t>
+          <t>2026-05-11 10:32:00</t>
         </is>
       </c>
       <c r="F517" t="inlineStr">
         <is>
-          <t>2026-05-11 09:42:00</t>
+          <t>2026-05-11 10:42:00</t>
         </is>
       </c>
       <c r="G517">
-        <v>24.92140864799025</v>
+        <v>25.84599396092362</v>
       </c>
       <c r="H517" t="inlineStr">
         <is>
@@ -21199,7 +21199,7 @@
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E519" t="inlineStr">
@@ -21271,7 +21271,7 @@
       </c>
       <c r="D521" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E521" t="inlineStr">
@@ -21343,7 +21343,7 @@
       </c>
       <c r="D523" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E523" t="inlineStr">
@@ -21415,7 +21415,7 @@
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E525" t="inlineStr">
@@ -21487,7 +21487,7 @@
       </c>
       <c r="D527" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E527" t="inlineStr">
@@ -21559,7 +21559,7 @@
       </c>
       <c r="D529" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E529" t="inlineStr">
@@ -21631,7 +21631,7 @@
       </c>
       <c r="D531" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E531" t="inlineStr">
@@ -21703,7 +21703,7 @@
       </c>
       <c r="D533" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E533" t="inlineStr">
@@ -21775,7 +21775,7 @@
       </c>
       <c r="D535" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E535" t="inlineStr">
@@ -21847,7 +21847,7 @@
       </c>
       <c r="D537" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E537" t="inlineStr">
@@ -21919,7 +21919,7 @@
       </c>
       <c r="D539" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E539" t="inlineStr">
@@ -21991,7 +21991,7 @@
       </c>
       <c r="D541" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E541" t="inlineStr">
@@ -22063,7 +22063,7 @@
       </c>
       <c r="D543" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E543" t="inlineStr">
@@ -22135,7 +22135,7 @@
       </c>
       <c r="D545" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E545" t="inlineStr">
@@ -22207,7 +22207,7 @@
       </c>
       <c r="D547" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E547" t="inlineStr">
@@ -22279,7 +22279,7 @@
       </c>
       <c r="D549" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E549" t="inlineStr">
@@ -22351,7 +22351,7 @@
       </c>
       <c r="D551" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E551" t="inlineStr">
@@ -22423,7 +22423,7 @@
       </c>
       <c r="D553" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E553" t="inlineStr">
@@ -22495,7 +22495,7 @@
       </c>
       <c r="D555" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E555" t="inlineStr">
@@ -22567,7 +22567,7 @@
       </c>
       <c r="D557" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E557" t="inlineStr">
@@ -22639,7 +22639,7 @@
       </c>
       <c r="D559" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E559" t="inlineStr">
@@ -22711,7 +22711,7 @@
       </c>
       <c r="D561" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E561" t="inlineStr">
@@ -22783,7 +22783,7 @@
       </c>
       <c r="D563" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E563" t="inlineStr">
@@ -22855,7 +22855,7 @@
       </c>
       <c r="D565" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E565" t="inlineStr">
@@ -22927,7 +22927,7 @@
       </c>
       <c r="D567" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E567" t="inlineStr">
@@ -22999,7 +22999,7 @@
       </c>
       <c r="D569" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E569" t="inlineStr">
@@ -23071,7 +23071,7 @@
       </c>
       <c r="D571" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E571" t="inlineStr">
@@ -23143,7 +23143,7 @@
       </c>
       <c r="D573" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E573" t="inlineStr">
@@ -23215,7 +23215,7 @@
       </c>
       <c r="D575" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E575" t="inlineStr">
@@ -23287,7 +23287,7 @@
       </c>
       <c r="D577" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E577" t="inlineStr">
@@ -23359,7 +23359,7 @@
       </c>
       <c r="D579" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E579" t="inlineStr">
@@ -23431,7 +23431,7 @@
       </c>
       <c r="D581" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E581" t="inlineStr">
@@ -23503,7 +23503,7 @@
       </c>
       <c r="D583" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E583" t="inlineStr">
@@ -23575,7 +23575,7 @@
       </c>
       <c r="D585" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E585" t="inlineStr">
@@ -23647,7 +23647,7 @@
       </c>
       <c r="D587" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E587" t="inlineStr">
@@ -23719,7 +23719,7 @@
       </c>
       <c r="D589" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E589" t="inlineStr">
@@ -23791,7 +23791,7 @@
       </c>
       <c r="D591" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E591" t="inlineStr">
@@ -23863,7 +23863,7 @@
       </c>
       <c r="D593" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E593" t="inlineStr">
@@ -23935,7 +23935,7 @@
       </c>
       <c r="D595" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E595" t="inlineStr">
@@ -24007,7 +24007,7 @@
       </c>
       <c r="D597" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E597" t="inlineStr">
@@ -24079,7 +24079,7 @@
       </c>
       <c r="D599" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E599" t="inlineStr">
@@ -24151,7 +24151,7 @@
       </c>
       <c r="D601" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E601" t="inlineStr">
@@ -24223,7 +24223,7 @@
       </c>
       <c r="D603" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E603" t="inlineStr">
@@ -24295,7 +24295,7 @@
       </c>
       <c r="D605" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E605" t="inlineStr">
@@ -24367,7 +24367,7 @@
       </c>
       <c r="D607" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E607" t="inlineStr">
@@ -24439,7 +24439,7 @@
       </c>
       <c r="D609" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E609" t="inlineStr">
@@ -24511,7 +24511,7 @@
       </c>
       <c r="D611" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E611" t="inlineStr">
@@ -24583,7 +24583,7 @@
       </c>
       <c r="D613" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E613" t="inlineStr">
@@ -24655,7 +24655,7 @@
       </c>
       <c r="D615" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E615" t="inlineStr">
@@ -24727,7 +24727,7 @@
       </c>
       <c r="D617" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E617" t="inlineStr">
@@ -24799,7 +24799,7 @@
       </c>
       <c r="D619" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E619" t="inlineStr">
@@ -24871,7 +24871,7 @@
       </c>
       <c r="D621" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E621" t="inlineStr">
@@ -24943,7 +24943,7 @@
       </c>
       <c r="D623" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E623" t="inlineStr">
@@ -25015,7 +25015,7 @@
       </c>
       <c r="D625" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E625" t="inlineStr">
@@ -25087,7 +25087,7 @@
       </c>
       <c r="D627" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E627" t="inlineStr">
@@ -25159,7 +25159,7 @@
       </c>
       <c r="D629" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E629" t="inlineStr">
@@ -25231,7 +25231,7 @@
       </c>
       <c r="D631" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E631" t="inlineStr">
@@ -25303,7 +25303,7 @@
       </c>
       <c r="D633" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E633" t="inlineStr">
@@ -25375,7 +25375,7 @@
       </c>
       <c r="D635" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E635" t="inlineStr">
@@ -25447,7 +25447,7 @@
       </c>
       <c r="D637" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E637" t="inlineStr">
@@ -25519,7 +25519,7 @@
       </c>
       <c r="D639" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E639" t="inlineStr">
@@ -25591,7 +25591,7 @@
       </c>
       <c r="D641" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E641" t="inlineStr">
@@ -25663,7 +25663,7 @@
       </c>
       <c r="D643" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E643" t="inlineStr">
@@ -25735,7 +25735,7 @@
       </c>
       <c r="D645" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E645" t="inlineStr">
@@ -25807,7 +25807,7 @@
       </c>
       <c r="D647" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E647" t="inlineStr">
@@ -25879,7 +25879,7 @@
       </c>
       <c r="D649" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E649" t="inlineStr">
@@ -25951,7 +25951,7 @@
       </c>
       <c r="D651" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E651" t="inlineStr">
@@ -26023,7 +26023,7 @@
       </c>
       <c r="D653" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E653" t="inlineStr">
@@ -26095,7 +26095,7 @@
       </c>
       <c r="D655" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E655" t="inlineStr">
@@ -26167,7 +26167,7 @@
       </c>
       <c r="D657" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E657" t="inlineStr">
@@ -26239,7 +26239,7 @@
       </c>
       <c r="D659" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E659" t="inlineStr">
@@ -26311,7 +26311,7 @@
       </c>
       <c r="D661" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E661" t="inlineStr">
@@ -26383,7 +26383,7 @@
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E663" t="inlineStr">
@@ -26455,7 +26455,7 @@
       </c>
       <c r="D665" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E665" t="inlineStr">
@@ -26527,7 +26527,7 @@
       </c>
       <c r="D667" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E667" t="inlineStr">
@@ -26599,7 +26599,7 @@
       </c>
       <c r="D669" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E669" t="inlineStr">
@@ -26671,7 +26671,7 @@
       </c>
       <c r="D671" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E671" t="inlineStr">
@@ -26743,7 +26743,7 @@
       </c>
       <c r="D673" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E673" t="inlineStr">
@@ -26815,7 +26815,7 @@
       </c>
       <c r="D675" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E675" t="inlineStr">
@@ -26887,7 +26887,7 @@
       </c>
       <c r="D677" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E677" t="inlineStr">
@@ -26959,7 +26959,7 @@
       </c>
       <c r="D679" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E679" t="inlineStr">
@@ -27031,7 +27031,7 @@
       </c>
       <c r="D681" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E681" t="inlineStr">
@@ -27103,7 +27103,7 @@
       </c>
       <c r="D683" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E683" t="inlineStr">
@@ -27175,7 +27175,7 @@
       </c>
       <c r="D685" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E685" t="inlineStr">
@@ -27247,7 +27247,7 @@
       </c>
       <c r="D687" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E687" t="inlineStr">
@@ -27319,7 +27319,7 @@
       </c>
       <c r="D689" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E689" t="inlineStr">
@@ -27360,16 +27360,16 @@
       </c>
       <c r="E690" t="inlineStr">
         <is>
-          <t>2026-05-24 12:17:02</t>
+          <t>2026-05-24 12:17:20</t>
         </is>
       </c>
       <c r="F690" t="inlineStr">
         <is>
-          <t>2026-05-24 12:27:02</t>
+          <t>2026-05-24 12:27:20</t>
         </is>
       </c>
       <c r="G690">
-        <v>25.5077344</v>
+        <v>25.509376</v>
       </c>
       <c r="H690" t="inlineStr">
         <is>
@@ -27391,7 +27391,7 @@
       </c>
       <c r="D691" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E691" t="inlineStr">
@@ -27463,7 +27463,7 @@
       </c>
       <c r="D693" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E693" t="inlineStr">
@@ -27535,7 +27535,7 @@
       </c>
       <c r="D695" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E695" t="inlineStr">
@@ -27607,7 +27607,7 @@
       </c>
       <c r="D697" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E697" t="inlineStr">
@@ -27679,7 +27679,7 @@
       </c>
       <c r="D699" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E699" t="inlineStr">
@@ -27751,7 +27751,7 @@
       </c>
       <c r="D701" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E701" t="inlineStr">
@@ -27823,7 +27823,7 @@
       </c>
       <c r="D703" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E703" t="inlineStr">
@@ -27895,7 +27895,7 @@
       </c>
       <c r="D705" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E705" t="inlineStr">
@@ -27967,7 +27967,7 @@
       </c>
       <c r="D707" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E707" t="inlineStr">
@@ -28039,7 +28039,7 @@
       </c>
       <c r="D709" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E709" t="inlineStr">
@@ -28111,7 +28111,7 @@
       </c>
       <c r="D711" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E711" t="inlineStr">
@@ -28183,7 +28183,7 @@
       </c>
       <c r="D713" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E713" t="inlineStr">
@@ -28255,7 +28255,7 @@
       </c>
       <c r="D715" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E715" t="inlineStr">
@@ -28327,7 +28327,7 @@
       </c>
       <c r="D717" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E717" t="inlineStr">
@@ -28399,7 +28399,7 @@
       </c>
       <c r="D719" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E719" t="inlineStr">
@@ -28471,7 +28471,7 @@
       </c>
       <c r="D721" t="inlineStr">
         <is>
-          <t>CO2_Fixation</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="E721" t="inlineStr">
@@ -28722,7 +28722,7 @@
       </c>
       <c r="E727" t="inlineStr">
         <is>
-          <t>2026-03-31 14:53:55</t>
+          <t>2026-03-31 13:53:55</t>
         </is>
       </c>
       <c r="F727" t="inlineStr">
@@ -28731,7 +28731,7 @@
         </is>
       </c>
       <c r="G727">
-        <v>26.6589</v>
+        <v>26.654</v>
       </c>
       <c r="H727" t="inlineStr">
         <is>
@@ -28739,10 +28739,10 @@
         </is>
       </c>
       <c r="I727">
-        <v>25.49784</v>
+        <v>23.44369</v>
       </c>
       <c r="J727">
-        <v>26.68006</v>
+        <v>26.67647</v>
       </c>
     </row>
     <row r="728">
@@ -35153,11 +35153,11 @@
       </c>
       <c r="F880" t="inlineStr">
         <is>
-          <t>2026-04-27 10:02:20</t>
+          <t>2026-04-27 12:02:20</t>
         </is>
       </c>
       <c r="G880">
-        <v>25.49775</v>
+        <v>25.5026</v>
       </c>
       <c r="H880" t="inlineStr">
         <is>
@@ -35165,10 +35165,10 @@
         </is>
       </c>
       <c r="I880">
-        <v>23.4863</v>
+        <v>24.5427</v>
       </c>
       <c r="J880">
-        <v>26.08023</v>
+        <v>26.6668</v>
       </c>
     </row>
     <row r="881">
@@ -40253,11 +40253,11 @@
       </c>
       <c r="F1018" t="inlineStr">
         <is>
-          <t>2026-05-17 02:12:50</t>
+          <t>2026-05-17 14:12:50</t>
         </is>
       </c>
       <c r="G1018">
-        <v>19.79721666666666</v>
+        <v>26.65925985130112</v>
       </c>
       <c r="H1018" t="inlineStr">
         <is>

</xml_diff>